<commit_message>
Accept your own invoice and payment CSVs with input validation; add 7 tests
</commit_message>
<xml_diff>
--- a/Sample_Payout_Reconciliation_Report.xlsx
+++ b/Sample_Payout_Reconciliation_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Adnan Desktop\Finance\payout-reconciliation-excel-report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22C0096-BA7E-44A9-8F91-0A67AA357FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1052978-D241-46D0-8450-CA8D74686CAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1077,7 +1077,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-7826-4A77-BF14-9EA730A3D18B}"/>
+                <c16:uniqueId val="{00000001-6BF2-436E-8BD2-9128DA07E35A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1098,7 +1098,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-7826-4A77-BF14-9EA730A3D18B}"/>
+                <c16:uniqueId val="{00000003-6BF2-436E-8BD2-9128DA07E35A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1119,7 +1119,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-7826-4A77-BF14-9EA730A3D18B}"/>
+                <c16:uniqueId val="{00000005-6BF2-436E-8BD2-9128DA07E35A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1140,7 +1140,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-7826-4A77-BF14-9EA730A3D18B}"/>
+                <c16:uniqueId val="{00000007-6BF2-436E-8BD2-9128DA07E35A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1161,7 +1161,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-7826-4A77-BF14-9EA730A3D18B}"/>
+                <c16:uniqueId val="{00000009-6BF2-436E-8BD2-9128DA07E35A}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1235,7 +1235,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000A-7826-4A77-BF14-9EA730A3D18B}"/>
+              <c16:uniqueId val="{0000000A-6BF2-436E-8BD2-9128DA07E35A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>